<commit_message>
S28 - plate-bearing test dictionaries, results, and DIN 18134 registry entry
Two new codelist dictionaries for PlateLoadTest/ZoneLoadTest
(loadingProcedure spanning ASTM D1196 nonrepetitive, ASTM D1195
repetitive and DIN 18134 two-cycle; plateStiffness). properties.xml
gains three result entries that were a genuine gap - modulus_of_
subgrade_reaction (ASTM's characteristic output) and deformation_
modulus_first_load/second_load (DIN 18134's Ev1/Ev2). measurementKind.xml
gains plate_load_test and zone_load_test (PI2), resolving the "PLT"/
"ZLT" abbreviation S6 had flagged and left unresolved. The registry
gains din_18134, the third governing-standard tradition for this test
family alongside the already-registered ASTM D1194 (already correctly
flagged withdrawn) and D1196.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/measurementKind.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/measurementKind.xlsx
@@ -1292,25 +1292,66 @@
     </row>
     <row r="9">
       <c r="A9" s="2">
-        <f>IF(ISNA(VLOOKUP(B9,AssociatedElements!B$2:B2947,1,FALSE)),"Not used","")</f>
-        <v/>
-      </c>
-      <c r="C9" s="16" t="n"/>
-      <c r="D9" s="16" t="n"/>
-      <c r="E9" s="17" t="n"/>
-      <c r="G9" s="9" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B9,AssociatedElements!B$2:B$999,1,FALSE)),"Not used","")</f>
+        <v/>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>plate_load_test</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Plate load test</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>A plate-bearing load test on a single deep foundation element head, measuring ground or platform stiffness rather than the element's own axial capacity, per ASTM D1194 (withdrawn 2003, still in practical use), ASTM D1195/D1196, or DIN 18134.</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>ASTM D1196</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2">
-        <f>IF(ISNA(VLOOKUP(B10,AssociatedElements!B$2:B2948,1,FALSE)),"Not used","")</f>
-        <v/>
-      </c>
-      <c r="B10" s="13" t="n"/>
-      <c r="C10" s="13" t="n"/>
-      <c r="D10" s="14" t="n"/>
-      <c r="E10" s="13" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B10,AssociatedElements!B$2:B$999,1,FALSE)),"Not used","")</f>
+        <v/>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>zone_load_test</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Zone load test</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>A large-plate load test on a load transfer platform over a group of columns, per BS 8006-1 (which requires the test), typically executed to ASTM D1195/D1196 or DIN 18134's methodology.</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F10" s="13" t="n"/>
-      <c r="G10" s="9" t="n"/>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>BS 8006-1</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2">
@@ -1785,17 +1826,35 @@
     </row>
     <row r="9">
       <c r="A9">
-        <f>IF(ISNA(VLOOKUP(B9,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B9" s="2" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B9,Definitions!B$2:B$999,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>plate_load_test</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>//diggs:TargetMeasurement/diggs:measurementKind</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10">
-        <f>IF(ISNA(VLOOKUP(B10,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B10" s="20" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B10,Definitions!B$2:B$999,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>zone_load_test</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>//diggs:TargetMeasurement/diggs:measurementKind</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11">

</xml_diff>